<commit_message>
Messprotokoll 1.0.0: Erfassung, Freigabe, Messmittel, Cpk-Auswertung, Installer
- Messung über Produktnummer mit Ampel, Zwischenspeichern, Abschließen, PDF
- n.i.O.-Entscheidungen mit Rollen (Nacharbeit/Sonderfreigabe/Ausschuss)
- Messmittelprüfung, offene Protokolle, Auswertung mit Cp/Cpk und Verlauf
- INSTALLIEREN.bat baut die .xlsm, Testdaten und Testplan für den großen Test
- Selbsttest in Excel; Tests in LibreOffice (Logik, Syntax, Deklarationen, Testdaten)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ApxXdbre9jhdnpctvqtjDG
</commit_message>
<xml_diff>
--- a/messprotokoll/dateien/Stammdaten.xlsx
+++ b/messprotokoll/dateien/Stammdaten.xlsx
@@ -13711,7 +13711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -13765,7 +13765,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Messmittel (wird in Phase 4 an die Erfassung angebunden)</t>
+          <t>Messmittel</t>
         </is>
       </c>
     </row>
@@ -13777,10 +13777,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr"/>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Abgelaufene Messmittel oder solche ohne Kalibrierdaten sind bei der Messung gesperrt.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Diese Datei darf nur die Stammdaten-Gruppe ändern (Ordnerrechte vom IT setzen lassen).</t>
         </is>

</xml_diff>